<commit_message>
auto: 05-08 23:05 | "export_example_\345\205\250\351\207\217.xlsx" "export_example_\346\214\211\346\234\210_2026-05.xlsx" scripts/gen_sample_xlsx.js src/utils/export.ts
</commit_message>
<xml_diff>
--- a/export_example_全量.xlsx
+++ b/export_example_全量.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="47">
   <si>
     <t>家教课程账单</t>
   </si>
@@ -90,7 +90,16 @@
     <t>待上课</t>
   </si>
   <si>
-    <t>合计: 4节课    8.0h    1160元    已收 600元 / 待收 560元</t>
+    <t>合计: 4节课</t>
+  </si>
+  <si>
+    <t>8.0h</t>
+  </si>
+  <si>
+    <t>1160元</t>
+  </si>
+  <si>
+    <t>已收 600元 / 待收 560元</t>
   </si>
   <si>
     <t>学生: 王雨涵    电话: 13801026789     英语 120元/h</t>
@@ -114,7 +123,16 @@
     <t>口语练习</t>
   </si>
   <si>
-    <t>合计: 2节课    4.0h    480元    已收 240元 / 待收 240元</t>
+    <t>合计: 2节课</t>
+  </si>
+  <si>
+    <t>4.0h</t>
+  </si>
+  <si>
+    <t>480元</t>
+  </si>
+  <si>
+    <t>已收 240元 / 待收 240元</t>
   </si>
   <si>
     <t>学生: 陈子豪    电话: 13701039876     数学 160元/h</t>
@@ -132,14 +150,17 @@
     <t>2026-05-08</t>
   </si>
   <si>
-    <t>合计: 2节课    4.0h    640元    已收 320元 / 待收 320元</t>
+    <t>640元</t>
+  </si>
+  <si>
+    <t>已收 320元 / 待收 320元</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -149,12 +170,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF1A1A2E"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <color rgb="FF4A4A6A"/>
-      <sz val="11"/>
     </font>
     <font>
       <b/>
@@ -191,11 +207,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -204,7 +219,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -546,15 +563,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -562,140 +570,149 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="B10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A10:G10"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -705,15 +722,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -721,94 +729,103 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>26</v>
+      <c r="A2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="A5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="4" t="s">
+      <c r="E5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="B6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>32</v>
+      <c r="E6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
+      <c r="A8" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A8:G8"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -818,15 +835,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -834,94 +842,103 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="G6" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="4" t="s">
+      <c r="B8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
+      <c r="E8" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A8:G8"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: 05-09 00:38 | "export_example_\345\205\250\351\207\217.xlsx" "export_example_\346\214\211\346\234\210_2026-05.xlsx" scripts/gen_sample_xlsx.js "~$export_example_\346\214\211\346\234\210_2026-05.xlsx"
</commit_message>
<xml_diff>
--- a/export_example_全量.xlsx
+++ b/export_example_全量.xlsx
@@ -88,15 +88,12 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -556,25 +553,25 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="str">
+      <c r="A10" s="2" t="str">
         <v>合计: 4节课</v>
       </c>
-      <c r="B10" s="5" t="str">
-        <v/>
-      </c>
-      <c r="C10" s="5" t="str">
-        <v/>
-      </c>
-      <c r="D10" s="5" t="str">
+      <c r="B10" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C10" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D10" s="2" t="str">
         <v>8.0h</v>
       </c>
-      <c r="E10" s="5" t="str">
+      <c r="E10" s="2" t="str">
         <v>1160元</v>
       </c>
-      <c r="F10" s="5" t="str">
+      <c r="F10" s="2" t="str">
         <v>已收 600元 / 待收 560元</v>
       </c>
-      <c r="G10" s="5" t="str">
+      <c r="G10" s="2" t="str">
         <v/>
       </c>
     </row>
@@ -669,25 +666,25 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="str">
+      <c r="A8" s="2" t="str">
         <v>合计: 2节课</v>
       </c>
-      <c r="B8" s="5" t="str">
-        <v/>
-      </c>
-      <c r="C8" s="5" t="str">
-        <v/>
-      </c>
-      <c r="D8" s="5" t="str">
+      <c r="B8" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D8" s="2" t="str">
         <v>4.0h</v>
       </c>
-      <c r="E8" s="5" t="str">
+      <c r="E8" s="2" t="str">
         <v>480元</v>
       </c>
-      <c r="F8" s="5" t="str">
+      <c r="F8" s="2" t="str">
         <v>已收 240元 / 待收 240元</v>
       </c>
-      <c r="G8" s="5" t="str">
+      <c r="G8" s="2" t="str">
         <v/>
       </c>
     </row>
@@ -782,25 +779,25 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="str">
+      <c r="A8" s="2" t="str">
         <v>合计: 2节课</v>
       </c>
-      <c r="B8" s="5" t="str">
-        <v/>
-      </c>
-      <c r="C8" s="5" t="str">
-        <v/>
-      </c>
-      <c r="D8" s="5" t="str">
+      <c r="B8" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D8" s="2" t="str">
         <v>4.0h</v>
       </c>
-      <c r="E8" s="5" t="str">
+      <c r="E8" s="2" t="str">
         <v>640元</v>
       </c>
-      <c r="F8" s="5" t="str">
+      <c r="F8" s="2" t="str">
         <v>已收 320元 / 待收 320元</v>
       </c>
-      <c r="G8" s="5" t="str">
+      <c r="G8" s="2" t="str">
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 05-09 01:28 | "export_example_\345\205\250\351\207\217.xlsx" "export_example_\346\214\211\346\234\210_2026-05.xlsx" scripts/gen_sample_xlsx.js src/utils/export.ts
</commit_message>
<xml_diff>
--- a/export_example_全量.xlsx
+++ b/export_example_全量.xlsx
@@ -35,7 +35,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -44,8 +44,28 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -64,6 +84,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFD1FAE5"/>
         <bgColor/>
       </patternFill>
@@ -71,6 +97,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFEF3C7"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD1FAE5"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -100,14 +132,18 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -456,7 +492,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>学生: 李小明    电话: 13901012345    数学 150元/h · 物理 130元/h</v>
       </c>
     </row>
@@ -484,48 +520,48 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="str">
+      <c r="A5" s="2" t="str">
         <v>2026-05-03</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="2" t="str">
         <v>数学</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="2" t="str">
         <v>09:00-11:00</v>
       </c>
-      <c r="D5" s="4" t="str">
+      <c r="D5" s="2" t="str">
         <v>2h</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="2" t="str">
         <v>300元</v>
       </c>
-      <c r="F5" s="4" t="str">
+      <c r="F5" s="2" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="2" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="str">
+      <c r="A6" s="2" t="str">
         <v>2026-05-05</v>
       </c>
-      <c r="B6" s="4" t="str">
+      <c r="B6" s="2" t="str">
         <v>数学</v>
       </c>
-      <c r="C6" s="4" t="str">
+      <c r="C6" s="2" t="str">
         <v>09:00-11:00</v>
       </c>
-      <c r="D6" s="4" t="str">
+      <c r="D6" s="2" t="str">
         <v>2h</v>
       </c>
-      <c r="E6" s="4" t="str">
+      <c r="E6" s="2" t="str">
         <v>300元</v>
       </c>
-      <c r="F6" s="4" t="str">
+      <c r="F6" s="2" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G6" s="4" t="str">
+      <c r="G6" s="2" t="str">
         <v/>
       </c>
     </row>
@@ -599,25 +635,25 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="str">
-        <v>合计: 4节课</v>
+      <c r="A11" s="6" t="str">
+        <v>合计:</v>
       </c>
       <c r="B11" s="2" t="str">
         <v/>
       </c>
-      <c r="C11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D11" s="2" t="str">
+      <c r="C11" s="6" t="str">
+        <v>4节</v>
+      </c>
+      <c r="D11" s="6" t="str">
         <v>8.0h</v>
       </c>
-      <c r="E11" s="2" t="str">
+      <c r="E11" s="6" t="str">
         <v>1160元</v>
       </c>
-      <c r="F11" s="4" t="str">
+      <c r="F11" s="7" t="str">
         <v>600元</v>
       </c>
-      <c r="G11" s="6" t="str">
+      <c r="G11" s="8" t="str">
         <v>560元</v>
       </c>
     </row>
@@ -647,7 +683,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>学生: 王雨涵    电话: 13801026789    英语 120元/h</v>
       </c>
     </row>
@@ -675,25 +711,25 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="str">
+      <c r="A5" s="2" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="2" t="str">
         <v>英语</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="2" t="str">
         <v>16:00-18:00</v>
       </c>
-      <c r="D5" s="4" t="str">
+      <c r="D5" s="2" t="str">
         <v>2h</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="2" t="str">
         <v>240元</v>
       </c>
-      <c r="F5" s="4" t="str">
+      <c r="F5" s="2" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="2" t="str">
         <v/>
       </c>
     </row>
@@ -736,33 +772,33 @@
       <c r="E8" s="2" t="str">
         <v/>
       </c>
-      <c r="F8" s="4" t="str">
+      <c r="F8" s="9" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G8" s="6" t="str">
+      <c r="G8" s="10" t="str">
         <v>待收款</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="str">
-        <v>合计: 2节课</v>
+      <c r="A9" s="6" t="str">
+        <v>合计:</v>
       </c>
       <c r="B9" s="2" t="str">
         <v/>
       </c>
-      <c r="C9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D9" s="2" t="str">
+      <c r="C9" s="6" t="str">
+        <v>2节</v>
+      </c>
+      <c r="D9" s="6" t="str">
         <v>4.0h</v>
       </c>
-      <c r="E9" s="2" t="str">
+      <c r="E9" s="6" t="str">
         <v>480元</v>
       </c>
-      <c r="F9" s="4" t="str">
+      <c r="F9" s="7" t="str">
         <v>240元</v>
       </c>
-      <c r="G9" s="6" t="str">
+      <c r="G9" s="8" t="str">
         <v>240元</v>
       </c>
     </row>
@@ -792,7 +828,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>学生: 陈子豪    电话: 13701039876    数学 160元/h</v>
       </c>
     </row>
@@ -820,25 +856,25 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="str">
+      <c r="A5" s="2" t="str">
         <v>2026-05-07</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="2" t="str">
         <v>数学</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="2" t="str">
         <v>10:00-12:00</v>
       </c>
-      <c r="D5" s="4" t="str">
+      <c r="D5" s="2" t="str">
         <v>2h</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="2" t="str">
         <v>320元</v>
       </c>
-      <c r="F5" s="4" t="str">
+      <c r="F5" s="2" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="2" t="str">
         <v/>
       </c>
     </row>
@@ -881,33 +917,33 @@
       <c r="E8" s="2" t="str">
         <v/>
       </c>
-      <c r="F8" s="4" t="str">
+      <c r="F8" s="9" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G8" s="6" t="str">
+      <c r="G8" s="10" t="str">
         <v>待收款</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="str">
-        <v>合计: 2节课</v>
+      <c r="A9" s="6" t="str">
+        <v>合计:</v>
       </c>
       <c r="B9" s="2" t="str">
         <v/>
       </c>
-      <c r="C9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D9" s="2" t="str">
+      <c r="C9" s="6" t="str">
+        <v>2节</v>
+      </c>
+      <c r="D9" s="6" t="str">
         <v>4.0h</v>
       </c>
-      <c r="E9" s="2" t="str">
+      <c r="E9" s="6" t="str">
         <v>640元</v>
       </c>
-      <c r="F9" s="4" t="str">
+      <c r="F9" s="7" t="str">
         <v>320元</v>
       </c>
-      <c r="G9" s="6" t="str">
+      <c r="G9" s="8" t="str">
         <v>320元</v>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 05-09 01:31 | "export_example_\345\205\250\351\207\217.xlsx" scripts/gen_sample_xlsx.js src/utils/export.ts
</commit_message>
<xml_diff>
--- a/export_example_全量.xlsx
+++ b/export_example_全量.xlsx
@@ -84,6 +84,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFD1FAE5"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFEF3C7"/>
         <bgColor/>
       </patternFill>
@@ -97,12 +103,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFEF3C7"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD1FAE5"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -139,10 +139,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles>
@@ -520,48 +520,48 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="str">
+      <c r="A5" s="4" t="str">
         <v>2026-05-03</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="5" t="str">
         <v>数学</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="5" t="str">
         <v>09:00-11:00</v>
       </c>
-      <c r="D5" s="2" t="str">
+      <c r="D5" s="5" t="str">
         <v>2h</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="5" t="str">
         <v>300元</v>
       </c>
-      <c r="F5" s="2" t="str">
+      <c r="F5" s="5" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G5" s="2" t="str">
+      <c r="G5" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="str">
+      <c r="A6" s="5" t="str">
         <v>2026-05-05</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="5" t="str">
         <v>数学</v>
       </c>
-      <c r="C6" s="2" t="str">
+      <c r="C6" s="5" t="str">
         <v>09:00-11:00</v>
       </c>
-      <c r="D6" s="2" t="str">
+      <c r="D6" s="5" t="str">
         <v>2h</v>
       </c>
-      <c r="E6" s="2" t="str">
+      <c r="E6" s="5" t="str">
         <v>300元</v>
       </c>
-      <c r="F6" s="2" t="str">
+      <c r="F6" s="5" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G6" s="2" t="str">
+      <c r="G6" s="5" t="str">
         <v/>
       </c>
     </row>
@@ -627,33 +627,33 @@
       <c r="E10" s="2" t="str">
         <v/>
       </c>
-      <c r="F10" s="4" t="str">
+      <c r="F10" s="5" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G10" s="5" t="str">
+      <c r="G10" s="6" t="str">
         <v>待收款</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="str">
+      <c r="A11" s="7" t="str">
         <v>合计:</v>
       </c>
       <c r="B11" s="2" t="str">
         <v/>
       </c>
-      <c r="C11" s="6" t="str">
+      <c r="C11" s="7" t="str">
         <v>4节</v>
       </c>
-      <c r="D11" s="6" t="str">
+      <c r="D11" s="7" t="str">
         <v>8.0h</v>
       </c>
-      <c r="E11" s="6" t="str">
+      <c r="E11" s="7" t="str">
         <v>1160元</v>
       </c>
-      <c r="F11" s="7" t="str">
+      <c r="F11" s="8" t="str">
         <v>600元</v>
       </c>
-      <c r="G11" s="8" t="str">
+      <c r="G11" s="9" t="str">
         <v>560元</v>
       </c>
     </row>
@@ -711,25 +711,25 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="str">
+      <c r="A5" s="5" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="5" t="str">
         <v>英语</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="5" t="str">
         <v>16:00-18:00</v>
       </c>
-      <c r="D5" s="2" t="str">
+      <c r="D5" s="5" t="str">
         <v>2h</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="5" t="str">
         <v>240元</v>
       </c>
-      <c r="F5" s="2" t="str">
+      <c r="F5" s="5" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G5" s="2" t="str">
+      <c r="G5" s="5" t="str">
         <v/>
       </c>
     </row>
@@ -772,7 +772,7 @@
       <c r="E8" s="2" t="str">
         <v/>
       </c>
-      <c r="F8" s="9" t="str">
+      <c r="F8" s="5" t="str">
         <v>✓ 已收款</v>
       </c>
       <c r="G8" s="10" t="str">
@@ -780,25 +780,25 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="str">
+      <c r="A9" s="7" t="str">
         <v>合计:</v>
       </c>
       <c r="B9" s="2" t="str">
         <v/>
       </c>
-      <c r="C9" s="6" t="str">
+      <c r="C9" s="7" t="str">
         <v>2节</v>
       </c>
-      <c r="D9" s="6" t="str">
+      <c r="D9" s="7" t="str">
         <v>4.0h</v>
       </c>
-      <c r="E9" s="6" t="str">
+      <c r="E9" s="7" t="str">
         <v>480元</v>
       </c>
-      <c r="F9" s="7" t="str">
+      <c r="F9" s="8" t="str">
         <v>240元</v>
       </c>
-      <c r="G9" s="8" t="str">
+      <c r="G9" s="9" t="str">
         <v>240元</v>
       </c>
     </row>
@@ -856,25 +856,25 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="str">
+      <c r="A5" s="5" t="str">
         <v>2026-05-07</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="5" t="str">
         <v>数学</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="5" t="str">
         <v>10:00-12:00</v>
       </c>
-      <c r="D5" s="2" t="str">
+      <c r="D5" s="5" t="str">
         <v>2h</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="5" t="str">
         <v>320元</v>
       </c>
-      <c r="F5" s="2" t="str">
+      <c r="F5" s="5" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G5" s="2" t="str">
+      <c r="G5" s="5" t="str">
         <v/>
       </c>
     </row>
@@ -917,7 +917,7 @@
       <c r="E8" s="2" t="str">
         <v/>
       </c>
-      <c r="F8" s="9" t="str">
+      <c r="F8" s="5" t="str">
         <v>✓ 已收款</v>
       </c>
       <c r="G8" s="10" t="str">
@@ -925,25 +925,25 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="str">
+      <c r="A9" s="7" t="str">
         <v>合计:</v>
       </c>
       <c r="B9" s="2" t="str">
         <v/>
       </c>
-      <c r="C9" s="6" t="str">
+      <c r="C9" s="7" t="str">
         <v>2节</v>
       </c>
-      <c r="D9" s="6" t="str">
+      <c r="D9" s="7" t="str">
         <v>4.0h</v>
       </c>
-      <c r="E9" s="6" t="str">
+      <c r="E9" s="7" t="str">
         <v>640元</v>
       </c>
-      <c r="F9" s="7" t="str">
+      <c r="F9" s="8" t="str">
         <v>320元</v>
       </c>
-      <c r="G9" s="8" t="str">
+      <c r="G9" s="9" t="str">
         <v>320元</v>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 05-09 01:51 | "export_example_\345\205\250\351\207\217.xlsx" "export_example_\346\214\211\346\234\210_2026-05.xlsx" scripts/gen_sample_xlsx.js src/utils/export.ts
</commit_message>
<xml_diff>
--- a/export_example_全量.xlsx
+++ b/export_example_全量.xlsx
@@ -35,7 +35,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -43,6 +43,12 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <name val="Calibri"/>
+      <b/>
+      <color rgb="0070C0"/>
     </font>
     <font>
       <sz val="14"/>
@@ -132,17 +138,18 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles>
@@ -487,12 +494,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
-        <v>家教课程账单</v>
+      <c r="A1" s="3" t="str">
+        <v>家教课程总账单</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="str">
+      <c r="A2" s="4" t="str">
         <v>学生: 李小明    电话: 13901012345    数学 150元/h · 物理 130元/h</v>
       </c>
     </row>
@@ -520,48 +527,48 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="str">
+      <c r="A5" s="5" t="str">
         <v>2026-05-03</v>
       </c>
-      <c r="B5" s="5" t="str">
+      <c r="B5" s="6" t="str">
         <v>数学</v>
       </c>
-      <c r="C5" s="5" t="str">
+      <c r="C5" s="6" t="str">
         <v>09:00-11:00</v>
       </c>
-      <c r="D5" s="5" t="str">
+      <c r="D5" s="6" t="str">
         <v>2h</v>
       </c>
-      <c r="E5" s="5" t="str">
+      <c r="E5" s="6" t="str">
         <v>300元</v>
       </c>
-      <c r="F5" s="5" t="str">
+      <c r="F5" s="6" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G5" s="5" t="str">
+      <c r="G5" s="6" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="str">
+      <c r="A6" s="6" t="str">
         <v>2026-05-05</v>
       </c>
-      <c r="B6" s="5" t="str">
+      <c r="B6" s="6" t="str">
         <v>数学</v>
       </c>
-      <c r="C6" s="5" t="str">
+      <c r="C6" s="6" t="str">
         <v>09:00-11:00</v>
       </c>
-      <c r="D6" s="5" t="str">
+      <c r="D6" s="6" t="str">
         <v>2h</v>
       </c>
-      <c r="E6" s="5" t="str">
+      <c r="E6" s="6" t="str">
         <v>300元</v>
       </c>
-      <c r="F6" s="5" t="str">
+      <c r="F6" s="6" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G6" s="5" t="str">
+      <c r="G6" s="6" t="str">
         <v/>
       </c>
     </row>
@@ -627,33 +634,33 @@
       <c r="E10" s="2" t="str">
         <v/>
       </c>
-      <c r="F10" s="5" t="str">
+      <c r="F10" s="6" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G10" s="6" t="str">
+      <c r="G10" s="7" t="str">
         <v>待收款</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="str">
+      <c r="A11" s="8" t="str">
         <v>合计:</v>
       </c>
       <c r="B11" s="2" t="str">
         <v/>
       </c>
-      <c r="C11" s="7" t="str">
+      <c r="C11" s="8" t="str">
         <v>4节</v>
       </c>
-      <c r="D11" s="7" t="str">
+      <c r="D11" s="8" t="str">
         <v>8.0h</v>
       </c>
-      <c r="E11" s="7" t="str">
+      <c r="E11" s="8" t="str">
         <v>1160元</v>
       </c>
-      <c r="F11" s="8" t="str">
+      <c r="F11" s="9" t="str">
         <v>600元</v>
       </c>
-      <c r="G11" s="9" t="str">
+      <c r="G11" s="10" t="str">
         <v>560元</v>
       </c>
     </row>
@@ -678,12 +685,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
-        <v>家教课程账单</v>
+      <c r="A1" s="3" t="str">
+        <v>家教课程总账单</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="str">
+      <c r="A2" s="4" t="str">
         <v>学生: 王雨涵    电话: 13801026789    英语 120元/h</v>
       </c>
     </row>
@@ -711,25 +718,25 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="str">
+      <c r="A5" s="6" t="str">
         <v>2026-05-04</v>
       </c>
-      <c r="B5" s="5" t="str">
+      <c r="B5" s="6" t="str">
         <v>英语</v>
       </c>
-      <c r="C5" s="5" t="str">
+      <c r="C5" s="6" t="str">
         <v>16:00-18:00</v>
       </c>
-      <c r="D5" s="5" t="str">
+      <c r="D5" s="6" t="str">
         <v>2h</v>
       </c>
-      <c r="E5" s="5" t="str">
+      <c r="E5" s="6" t="str">
         <v>240元</v>
       </c>
-      <c r="F5" s="5" t="str">
+      <c r="F5" s="6" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G5" s="5" t="str">
+      <c r="G5" s="6" t="str">
         <v/>
       </c>
     </row>
@@ -772,33 +779,33 @@
       <c r="E8" s="2" t="str">
         <v/>
       </c>
-      <c r="F8" s="5" t="str">
+      <c r="F8" s="6" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G8" s="10" t="str">
+      <c r="G8" s="11" t="str">
         <v>待收款</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="str">
+      <c r="A9" s="8" t="str">
         <v>合计:</v>
       </c>
       <c r="B9" s="2" t="str">
         <v/>
       </c>
-      <c r="C9" s="7" t="str">
+      <c r="C9" s="8" t="str">
         <v>2节</v>
       </c>
-      <c r="D9" s="7" t="str">
+      <c r="D9" s="8" t="str">
         <v>4.0h</v>
       </c>
-      <c r="E9" s="7" t="str">
+      <c r="E9" s="8" t="str">
         <v>480元</v>
       </c>
-      <c r="F9" s="8" t="str">
+      <c r="F9" s="9" t="str">
         <v>240元</v>
       </c>
-      <c r="G9" s="9" t="str">
+      <c r="G9" s="10" t="str">
         <v>240元</v>
       </c>
     </row>
@@ -823,12 +830,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
-        <v>家教课程账单</v>
+      <c r="A1" s="3" t="str">
+        <v>家教课程总账单</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="str">
+      <c r="A2" s="4" t="str">
         <v>学生: 陈子豪    电话: 13701039876    数学 160元/h</v>
       </c>
     </row>
@@ -856,25 +863,25 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="str">
+      <c r="A5" s="6" t="str">
         <v>2026-05-07</v>
       </c>
-      <c r="B5" s="5" t="str">
+      <c r="B5" s="6" t="str">
         <v>数学</v>
       </c>
-      <c r="C5" s="5" t="str">
+      <c r="C5" s="6" t="str">
         <v>10:00-12:00</v>
       </c>
-      <c r="D5" s="5" t="str">
+      <c r="D5" s="6" t="str">
         <v>2h</v>
       </c>
-      <c r="E5" s="5" t="str">
+      <c r="E5" s="6" t="str">
         <v>320元</v>
       </c>
-      <c r="F5" s="5" t="str">
+      <c r="F5" s="6" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G5" s="5" t="str">
+      <c r="G5" s="6" t="str">
         <v/>
       </c>
     </row>
@@ -917,33 +924,33 @@
       <c r="E8" s="2" t="str">
         <v/>
       </c>
-      <c r="F8" s="5" t="str">
+      <c r="F8" s="6" t="str">
         <v>✓ 已收款</v>
       </c>
-      <c r="G8" s="10" t="str">
+      <c r="G8" s="11" t="str">
         <v>待收款</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="str">
+      <c r="A9" s="8" t="str">
         <v>合计:</v>
       </c>
       <c r="B9" s="2" t="str">
         <v/>
       </c>
-      <c r="C9" s="7" t="str">
+      <c r="C9" s="8" t="str">
         <v>2节</v>
       </c>
-      <c r="D9" s="7" t="str">
+      <c r="D9" s="8" t="str">
         <v>4.0h</v>
       </c>
-      <c r="E9" s="7" t="str">
+      <c r="E9" s="8" t="str">
         <v>640元</v>
       </c>
-      <c r="F9" s="8" t="str">
+      <c r="F9" s="9" t="str">
         <v>320元</v>
       </c>
-      <c r="G9" s="9" t="str">
+      <c r="G9" s="10" t="str">
         <v>320元</v>
       </c>
     </row>

</xml_diff>